<commit_message>
Update course status handling and sorting logic in course-list.html
</commit_message>
<xml_diff>
--- a/course_list.xlsx
+++ b/course_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://4spe-my.sharepoint.com/personal/pmatos_4spe_org/Documents/ee--Events/01--SPE Academy/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://4spe-my.sharepoint.com/personal/pmatos_4spe_org/Documents/ee--Events/01--SPE Academy/Online Courses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="14_{F278B288-687A-0B4F-B5D3-A8AB2DF815F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80EE7663-FAA2-D44C-A647-FFE6CFE7B33B}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="14_{F278B288-687A-0B4F-B5D3-A8AB2DF815F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CB8BD46-2905-C744-8A2F-D1ED46E2E60D}"/>
   <bookViews>
-    <workbookView xWindow="4480" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{58D91B09-677B-7B46-89F6-C0AC19DB45D7}"/>
+    <workbookView xWindow="4480" yWindow="660" windowWidth="30920" windowHeight="20360" xr2:uid="{58D91B09-677B-7B46-89F6-C0AC19DB45D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="98">
   <si>
     <t>course_id</t>
   </si>
@@ -62,42 +62,18 @@
     <t>total_hours</t>
   </si>
   <si>
-    <t>online_bool</t>
-  </si>
-  <si>
-    <t>pricing</t>
-  </si>
-  <si>
     <t>course_url</t>
   </si>
   <si>
     <t>course_img_src</t>
   </si>
   <si>
-    <t>course_description</t>
-  </si>
-  <si>
-    <t>course_rating</t>
-  </si>
-  <si>
-    <t>{'Premium': '$720', 'Members': '$800', 'Nonmembers': '$1000'}</t>
-  </si>
-  <si>
     <t>Intermediate</t>
   </si>
   <si>
-    <t>{'Premium': '$540', 'Members': '$600', 'Nonmembers': '$800'}</t>
-  </si>
-  <si>
     <t>Jeffrey A. Jensen</t>
   </si>
   <si>
-    <t>{'Premium': 'Free', 'Members': '$49', 'Student Members': '$25', 'Nonmembers': '$249'}</t>
-  </si>
-  <si>
-    <t>{'Premium': '$360', 'Members': '$400', 'Nonmembers': '$600'}</t>
-  </si>
-  <si>
     <t>Consider Recycling when Addressing Polymer Design and Optimization</t>
   </si>
   <si>
@@ -305,9 +281,6 @@
     <t>/i4a/pages/index.cfm?pageID=9003</t>
   </si>
   <si>
-    <t>{'All Attendees': 'Free'}</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sammi Sadler &amp; Stephanie Williams </t>
   </si>
   <si>
@@ -326,9 +299,6 @@
     <t>PFAS</t>
   </si>
   <si>
-    <t>{'Premium': 'Free', 'Members': '$49', 'Nonmembers': '$249'}</t>
-  </si>
-  <si>
     <t>/i4a/pages/index.cfm?pageID=9285</t>
   </si>
   <si>
@@ -351,6 +321,15 @@
   </si>
   <si>
     <t>/images/events/2025/ww--courses/course-bio-plasticizers-for-pvc.webp</t>
+  </si>
+  <si>
+    <t>course_status</t>
+  </si>
+  <si>
+    <t>ondemand</t>
+  </si>
+  <si>
+    <t>online</t>
   </si>
 </sst>
 </file>
@@ -490,12 +469,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{96A166DF-A472-3B4B-9904-36C62EC18415}" name="Table1" displayName="Table1" ref="A1:O21" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:O21" xr:uid="{96A166DF-A472-3B4B-9904-36C62EC18415}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{96A166DF-A472-3B4B-9904-36C62EC18415}" name="Table1" displayName="Table1" ref="A1:L21" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:L21" xr:uid="{96A166DF-A472-3B4B-9904-36C62EC18415}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L9">
     <sortCondition ref="B1:B9"/>
   </sortState>
-  <tableColumns count="15">
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{8A686DFE-D88F-B94C-9D90-C0734D5CC5A8}" name="course_id"/>
     <tableColumn id="2" xr3:uid="{04FE514E-57B7-4D42-8290-3FED320837C5}" name="course_start_date" dataDxfId="2"/>
     <tableColumn id="15" xr3:uid="{44474086-7966-9541-AE0F-4B389D207EEC}" name="course_end_date" dataDxfId="1"/>
@@ -505,12 +484,9 @@
     <tableColumn id="6" xr3:uid="{9692E90B-4059-A949-8145-5383BE222A95}" name="course_level"/>
     <tableColumn id="7" xr3:uid="{E5F7F0E1-0051-5C44-A2D1-2EA4C5948E29}" name="total_sessions"/>
     <tableColumn id="8" xr3:uid="{A1071AC6-254E-BC45-8573-9ABD912DA571}" name="total_hours"/>
-    <tableColumn id="9" xr3:uid="{0E6DDF6F-C320-0A4A-A138-3DC67EEE466F}" name="online_bool"/>
-    <tableColumn id="10" xr3:uid="{862B5B94-9EA9-4742-8606-BFA8A8B0FDFC}" name="pricing"/>
+    <tableColumn id="9" xr3:uid="{0E6DDF6F-C320-0A4A-A138-3DC67EEE466F}" name="course_status"/>
     <tableColumn id="11" xr3:uid="{DBCD19B7-39A6-8848-B79A-63AC1EE1A4D0}" name="course_url"/>
     <tableColumn id="12" xr3:uid="{925AFC37-886C-1644-A47C-9359851D8F89}" name="course_img_src"/>
-    <tableColumn id="13" xr3:uid="{F1D8E5B8-B0E3-114C-A02C-D4C628D3619C}" name="course_description"/>
-    <tableColumn id="14" xr3:uid="{FABC5319-4353-BD49-A5DF-5E950F0DC395}" name="course_rating"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -833,7 +809,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F602E3B9-8D43-AE4F-B90E-B1B2D7D0B179}">
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5" customWidth="1"/>
@@ -844,14 +820,11 @@
     <col min="7" max="7" width="13.83203125" customWidth="1"/>
     <col min="8" max="8" width="15.6640625" customWidth="1"/>
     <col min="9" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="68.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="47.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="89" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.33203125" customWidth="1"/>
-    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="47.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="89" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -859,7 +832,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>2</v>
@@ -880,26 +853,17 @@
         <v>7</v>
       </c>
       <c r="J1" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="4"/>
-    </row>
-    <row r="2" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M1" s="4"/>
+    </row>
+    <row r="2" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>11</v>
       </c>
@@ -910,16 +874,16 @@
         <v>45632</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -927,20 +891,17 @@
       <c r="I2">
         <v>1</v>
       </c>
-      <c r="J2" t="b">
-        <v>1</v>
-      </c>
-      <c r="K2" t="s">
-        <v>18</v>
+      <c r="J2" t="s">
+        <v>96</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>45</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>12</v>
       </c>
@@ -951,16 +912,16 @@
         <v>45714</v>
       </c>
       <c r="D3" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H3">
         <v>4</v>
@@ -968,20 +929,17 @@
       <c r="I3">
         <v>4</v>
       </c>
-      <c r="J3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K3" t="s">
-        <v>19</v>
+      <c r="J3" t="s">
+        <v>97</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>46</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>13</v>
       </c>
@@ -992,16 +950,16 @@
         <v>45696</v>
       </c>
       <c r="D4" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="F4" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H4">
         <v>4</v>
@@ -1009,20 +967,17 @@
       <c r="I4">
         <v>4</v>
       </c>
-      <c r="J4" t="b">
-        <v>1</v>
-      </c>
-      <c r="K4" t="s">
-        <v>19</v>
+      <c r="J4" t="s">
+        <v>96</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>47</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>14</v>
       </c>
@@ -1033,16 +988,16 @@
         <v>45703</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F5" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H5">
         <v>4</v>
@@ -1050,20 +1005,17 @@
       <c r="I5">
         <v>4</v>
       </c>
-      <c r="J5" t="b">
-        <v>1</v>
-      </c>
-      <c r="K5" t="s">
-        <v>19</v>
+      <c r="J5" t="s">
+        <v>96</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>15</v>
       </c>
@@ -1074,16 +1026,16 @@
         <v>45743</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="G6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H6">
         <v>4</v>
@@ -1091,20 +1043,17 @@
       <c r="I6">
         <v>8</v>
       </c>
-      <c r="J6" t="b">
-        <v>1</v>
-      </c>
-      <c r="K6" t="s">
-        <v>14</v>
+      <c r="J6" t="s">
+        <v>97</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>16</v>
       </c>
@@ -1115,16 +1064,16 @@
         <v>45748</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="G7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H7">
         <v>3</v>
@@ -1132,20 +1081,17 @@
       <c r="I7">
         <v>6</v>
       </c>
-      <c r="J7" t="b">
-        <v>1</v>
-      </c>
-      <c r="K7" t="s">
-        <v>16</v>
+      <c r="J7" t="s">
+        <v>97</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>17</v>
       </c>
@@ -1156,16 +1102,16 @@
         <v>45765</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F8" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H8">
         <v>4</v>
@@ -1173,20 +1119,17 @@
       <c r="I8">
         <v>8</v>
       </c>
-      <c r="J8" t="b">
-        <v>1</v>
-      </c>
-      <c r="K8" t="s">
-        <v>14</v>
+      <c r="J8" t="s">
+        <v>97</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>51</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>18</v>
       </c>
@@ -1197,16 +1140,16 @@
         <v>45799</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H9">
         <v>4</v>
@@ -1214,20 +1157,17 @@
       <c r="I9">
         <v>6</v>
       </c>
-      <c r="J9" t="b">
-        <v>1</v>
-      </c>
-      <c r="K9" t="s">
-        <v>16</v>
+      <c r="J9" t="s">
+        <v>97</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>19</v>
       </c>
@@ -1238,16 +1178,16 @@
         <v>45681</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -1255,20 +1195,17 @@
       <c r="I10">
         <v>1</v>
       </c>
-      <c r="J10" t="b">
-        <v>1</v>
+      <c r="J10" t="s">
+        <v>96</v>
       </c>
       <c r="K10" t="s">
-        <v>18</v>
-      </c>
-      <c r="L10" t="s">
-        <v>61</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>20</v>
       </c>
@@ -1279,16 +1216,16 @@
         <v>45941</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F11" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G11" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -1296,20 +1233,17 @@
       <c r="I11">
         <v>1</v>
       </c>
-      <c r="J11" t="b">
-        <v>1</v>
-      </c>
-      <c r="K11" t="s">
-        <v>18</v>
+      <c r="J11" t="s">
+        <v>97</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>21</v>
       </c>
@@ -1320,16 +1254,16 @@
         <v>45980</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="E12" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G12" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -1337,20 +1271,17 @@
       <c r="I12">
         <v>1</v>
       </c>
-      <c r="J12" t="b">
-        <v>1</v>
-      </c>
-      <c r="K12" t="s">
-        <v>18</v>
+      <c r="J12" t="s">
+        <v>97</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>55</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="M12" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>22</v>
       </c>
@@ -1361,16 +1292,16 @@
         <v>45792</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E13" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F13" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G13" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H13">
         <v>1</v>
@@ -1378,20 +1309,17 @@
       <c r="I13">
         <v>1</v>
       </c>
-      <c r="J13" t="b">
-        <v>1</v>
-      </c>
-      <c r="K13" t="s">
-        <v>18</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="M13" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J13" t="s">
+        <v>97</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L13" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>23</v>
       </c>
@@ -1402,16 +1330,16 @@
         <v>45996</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E14" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F14" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -1419,20 +1347,17 @@
       <c r="I14">
         <v>1</v>
       </c>
-      <c r="J14" t="b">
-        <v>1</v>
-      </c>
-      <c r="K14" t="s">
-        <v>18</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="M14" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J14" t="s">
+        <v>97</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="L14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>24</v>
       </c>
@@ -1443,16 +1368,16 @@
         <v>45708</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F15" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="G15" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -1460,20 +1385,17 @@
       <c r="I15">
         <v>1</v>
       </c>
-      <c r="J15" t="b">
-        <v>1</v>
-      </c>
-      <c r="K15" t="s">
-        <v>18</v>
+      <c r="J15" t="s">
+        <v>97</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>58</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M15" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>25</v>
       </c>
@@ -1484,16 +1406,16 @@
         <v>45730</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="E16" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F16" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="G16" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -1501,20 +1423,17 @@
       <c r="I16">
         <v>1</v>
       </c>
-      <c r="J16" t="b">
-        <v>1</v>
-      </c>
-      <c r="K16" t="s">
-        <v>18</v>
+      <c r="J16" t="s">
+        <v>97</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="M16" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>26</v>
       </c>
@@ -1525,16 +1444,16 @@
         <v>45905</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="E17" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F17" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="G17" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H17">
         <v>1</v>
@@ -1542,20 +1461,17 @@
       <c r="I17">
         <v>1</v>
       </c>
-      <c r="J17" t="b">
-        <v>1</v>
-      </c>
-      <c r="K17" t="s">
-        <v>18</v>
+      <c r="J17" t="s">
+        <v>97</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>60</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="M17" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>27</v>
       </c>
@@ -1566,16 +1482,16 @@
         <v>45911</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="E18" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="F18" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G18" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H18">
         <v>4</v>
@@ -1583,20 +1499,17 @@
       <c r="I18">
         <v>8</v>
       </c>
-      <c r="J18" t="b">
-        <v>1</v>
-      </c>
-      <c r="K18" t="s">
-        <v>14</v>
-      </c>
-      <c r="L18" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="M18" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J18" t="s">
+        <v>97</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="L18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>28</v>
       </c>
@@ -1607,16 +1520,16 @@
         <v>45700</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="F19" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G19" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H19">
         <v>1</v>
@@ -1624,20 +1537,17 @@
       <c r="I19">
         <v>1</v>
       </c>
-      <c r="J19" t="b">
-        <v>1</v>
+      <c r="J19" t="s">
+        <v>97</v>
       </c>
       <c r="K19" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="L19" t="s">
-        <v>88</v>
-      </c>
-      <c r="M19" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>29</v>
       </c>
@@ -1648,16 +1558,16 @@
         <v>45757</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="E20" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="F20" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="G20" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -1665,20 +1575,17 @@
       <c r="I20">
         <v>1</v>
       </c>
-      <c r="J20" t="b">
-        <v>1</v>
+      <c r="J20" t="s">
+        <v>97</v>
       </c>
       <c r="K20" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="L20" t="s">
-        <v>97</v>
-      </c>
-      <c r="M20" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>30</v>
       </c>
@@ -1689,16 +1596,16 @@
         <v>45737</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="E21" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F21" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="G21" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="H21">
         <v>1</v>
@@ -1706,48 +1613,45 @@
       <c r="I21">
         <v>1</v>
       </c>
-      <c r="J21" t="b">
-        <v>1</v>
+      <c r="J21" t="s">
+        <v>97</v>
       </c>
       <c r="K21" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L21" t="s">
-        <v>103</v>
-      </c>
-      <c r="M21" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="L9" r:id="rId1" display="https://www.4spe.org/i4a/pages/index.cfm?pageid=8850" xr:uid="{C28AE2EB-D073-AB43-8BD8-95CD8337164E}"/>
-    <hyperlink ref="L2" r:id="rId2" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=8575" xr:uid="{A2C84F15-9228-C04A-8446-85AB232663EB}"/>
-    <hyperlink ref="M2" r:id="rId3" display="https://www.4spe.org/images/events/2023/webinar/webinar-dma-12-catalog.jpg" xr:uid="{2EC7FC7A-FB03-E34B-A223-47EEE6F03FBB}"/>
-    <hyperlink ref="L3" r:id="rId4" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9144" xr:uid="{181C4631-C7DA-B447-A42E-31EF545DBB60}"/>
-    <hyperlink ref="M3" r:id="rId5" display="https://www.4spe.org/images/events/2024/workshop/spe-course-troubleshooting-injection-molding.webp" xr:uid="{77EC2CAC-B1CB-E64C-A036-0E94E10D9703}"/>
-    <hyperlink ref="L4" r:id="rId6" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9150" xr:uid="{FD0C74D4-BB83-7447-AC15-B059808330E3}"/>
-    <hyperlink ref="M4" r:id="rId7" display="https://www.4spe.org/images/events/2024/workshop/spe-course-material-suggestion-catalog.webp" xr:uid="{31DDE21D-A296-6047-9FED-6C0823F77774}"/>
-    <hyperlink ref="L5" r:id="rId8" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=8210" xr:uid="{BE64A64A-D0D7-884D-A354-A27F95A79E93}"/>
-    <hyperlink ref="M5" r:id="rId9" display="https://www.4spe.org/images/events/2024/workshop/spe-course-troubleshooting-extrusion-catalog.webp" xr:uid="{58288FA1-CB79-3941-BDC1-37FEAA28F552}"/>
-    <hyperlink ref="L7" r:id="rId10" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9182" xr:uid="{FD243456-6274-0E4C-9248-DE59674C1F70}"/>
-    <hyperlink ref="M7" r:id="rId11" display="https://www.4spe.org/images/events/event-catalog/spe-workshop-material-recycling.webp?ver=2" xr:uid="{4C90A90C-4662-B846-8808-389977C64895}"/>
-    <hyperlink ref="M8" r:id="rId12" display="https://www.4spe.org/images/events/event-catalog/worshop-plastic-additives.webp?ver=2" xr:uid="{FAD81F91-F667-FA4A-A9EA-80BECFC024AC}"/>
-    <hyperlink ref="M6" r:id="rId13" display="https://www.4spe.org/images/events/2024/workshop/workshop-failure-in-plastics(1).jpg?ver=2" xr:uid="{54041E0A-7C4A-654B-A1F8-1985B9CDEA6E}"/>
-    <hyperlink ref="M10" r:id="rId14" display="https://www.4spe.org/images/events/2025/ww--courses/course-fourier-analysis.webp" xr:uid="{7AA8F333-96C5-DE4B-8F36-FC973038016B}"/>
-    <hyperlink ref="L11" r:id="rId15" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9209" xr:uid="{C423F1D5-089F-B54F-997C-03479C8204F5}"/>
-    <hyperlink ref="M11" r:id="rId16" display="https://www.4spe.org/images/events/2025/ww--courses/course-polymer-molecular-weight.webp" xr:uid="{DE1854BF-1713-C64F-A1D5-7E22202E899E}"/>
-    <hyperlink ref="M12" r:id="rId17" display="https://www.4spe.org/images/events/2025/ww--courses/course-thermal-dependency-of-plastics.webp" xr:uid="{6114DB1F-224C-4740-B48F-C2E19807BFBF}"/>
-    <hyperlink ref="L12" r:id="rId18" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9212" xr:uid="{B3D3C419-0FC0-634D-9DB3-8C5E21392085}"/>
-    <hyperlink ref="L13" r:id="rId19" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=7136" xr:uid="{674C115C-9B91-4A42-8CCF-31C01D77981E}"/>
-    <hyperlink ref="L14" r:id="rId20" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9215" xr:uid="{F9B3C5F5-8E5F-4049-9535-2D0FB4BC0108}"/>
-    <hyperlink ref="L15" r:id="rId21" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=6226" xr:uid="{DEB06038-3058-8245-A51D-FEB2BD91CD75}"/>
-    <hyperlink ref="M15" r:id="rId22" display="https://www.4spe.org/images/events/2025/ww--courses/course-navigating-material-selection.webp" xr:uid="{ED3E0BC8-FB56-4041-9302-46F97618FFCE}"/>
-    <hyperlink ref="L16" r:id="rId23" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=7134" xr:uid="{877E8FBD-E236-5A41-8319-3CAE7BB5D345}"/>
-    <hyperlink ref="M16" r:id="rId24" display="https://www.4spe.org/images/events/2025/ww--courses/course-rubber-o-rings-thumb.webp" xr:uid="{B2B08EFB-49AB-524D-8064-5B8FDBC69BEE}"/>
-    <hyperlink ref="M17" r:id="rId25" display="https://www.4spe.org/images/events/2025/ww--courses/course-chemical-resistance-of-palstics.webp" xr:uid="{2F193417-2F4B-914A-9FF3-2E279492ADE3}"/>
-    <hyperlink ref="L17" r:id="rId26" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9218" xr:uid="{E0F4DB60-6B6A-334B-B149-2B7869538B50}"/>
-    <hyperlink ref="L18" r:id="rId27" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9239" xr:uid="{061FEADD-FD12-224D-BBEB-9E560D7996A9}"/>
+    <hyperlink ref="K9" r:id="rId1" display="https://www.4spe.org/i4a/pages/index.cfm?pageid=8850" xr:uid="{C28AE2EB-D073-AB43-8BD8-95CD8337164E}"/>
+    <hyperlink ref="K2" r:id="rId2" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=8575" xr:uid="{A2C84F15-9228-C04A-8446-85AB232663EB}"/>
+    <hyperlink ref="L2" r:id="rId3" display="https://www.4spe.org/images/events/2023/webinar/webinar-dma-12-catalog.jpg" xr:uid="{2EC7FC7A-FB03-E34B-A223-47EEE6F03FBB}"/>
+    <hyperlink ref="K3" r:id="rId4" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9144" xr:uid="{181C4631-C7DA-B447-A42E-31EF545DBB60}"/>
+    <hyperlink ref="L3" r:id="rId5" display="https://www.4spe.org/images/events/2024/workshop/spe-course-troubleshooting-injection-molding.webp" xr:uid="{77EC2CAC-B1CB-E64C-A036-0E94E10D9703}"/>
+    <hyperlink ref="K4" r:id="rId6" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9150" xr:uid="{FD0C74D4-BB83-7447-AC15-B059808330E3}"/>
+    <hyperlink ref="L4" r:id="rId7" display="https://www.4spe.org/images/events/2024/workshop/spe-course-material-suggestion-catalog.webp" xr:uid="{31DDE21D-A296-6047-9FED-6C0823F77774}"/>
+    <hyperlink ref="K5" r:id="rId8" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=8210" xr:uid="{BE64A64A-D0D7-884D-A354-A27F95A79E93}"/>
+    <hyperlink ref="L5" r:id="rId9" display="https://www.4spe.org/images/events/2024/workshop/spe-course-troubleshooting-extrusion-catalog.webp" xr:uid="{58288FA1-CB79-3941-BDC1-37FEAA28F552}"/>
+    <hyperlink ref="K7" r:id="rId10" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9182" xr:uid="{FD243456-6274-0E4C-9248-DE59674C1F70}"/>
+    <hyperlink ref="L7" r:id="rId11" display="https://www.4spe.org/images/events/event-catalog/spe-workshop-material-recycling.webp?ver=2" xr:uid="{4C90A90C-4662-B846-8808-389977C64895}"/>
+    <hyperlink ref="L8" r:id="rId12" display="https://www.4spe.org/images/events/event-catalog/worshop-plastic-additives.webp?ver=2" xr:uid="{FAD81F91-F667-FA4A-A9EA-80BECFC024AC}"/>
+    <hyperlink ref="L6" r:id="rId13" display="https://www.4spe.org/images/events/2024/workshop/workshop-failure-in-plastics(1).jpg?ver=2" xr:uid="{54041E0A-7C4A-654B-A1F8-1985B9CDEA6E}"/>
+    <hyperlink ref="L10" r:id="rId14" display="https://www.4spe.org/images/events/2025/ww--courses/course-fourier-analysis.webp" xr:uid="{7AA8F333-96C5-DE4B-8F36-FC973038016B}"/>
+    <hyperlink ref="K11" r:id="rId15" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9209" xr:uid="{C423F1D5-089F-B54F-997C-03479C8204F5}"/>
+    <hyperlink ref="L11" r:id="rId16" display="https://www.4spe.org/images/events/2025/ww--courses/course-polymer-molecular-weight.webp" xr:uid="{DE1854BF-1713-C64F-A1D5-7E22202E899E}"/>
+    <hyperlink ref="L12" r:id="rId17" display="https://www.4spe.org/images/events/2025/ww--courses/course-thermal-dependency-of-plastics.webp" xr:uid="{6114DB1F-224C-4740-B48F-C2E19807BFBF}"/>
+    <hyperlink ref="K12" r:id="rId18" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9212" xr:uid="{B3D3C419-0FC0-634D-9DB3-8C5E21392085}"/>
+    <hyperlink ref="K13" r:id="rId19" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=7136" xr:uid="{674C115C-9B91-4A42-8CCF-31C01D77981E}"/>
+    <hyperlink ref="K14" r:id="rId20" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9215" xr:uid="{F9B3C5F5-8E5F-4049-9535-2D0FB4BC0108}"/>
+    <hyperlink ref="K15" r:id="rId21" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=6226" xr:uid="{DEB06038-3058-8245-A51D-FEB2BD91CD75}"/>
+    <hyperlink ref="L15" r:id="rId22" display="https://www.4spe.org/images/events/2025/ww--courses/course-navigating-material-selection.webp" xr:uid="{ED3E0BC8-FB56-4041-9302-46F97618FFCE}"/>
+    <hyperlink ref="K16" r:id="rId23" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=7134" xr:uid="{877E8FBD-E236-5A41-8319-3CAE7BB5D345}"/>
+    <hyperlink ref="L16" r:id="rId24" display="https://www.4spe.org/images/events/2025/ww--courses/course-rubber-o-rings-thumb.webp" xr:uid="{B2B08EFB-49AB-524D-8064-5B8FDBC69BEE}"/>
+    <hyperlink ref="L17" r:id="rId25" display="https://www.4spe.org/images/events/2025/ww--courses/course-chemical-resistance-of-palstics.webp" xr:uid="{2F193417-2F4B-914A-9FF3-2E279492ADE3}"/>
+    <hyperlink ref="K17" r:id="rId26" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9218" xr:uid="{E0F4DB60-6B6A-334B-B149-2B7869538B50}"/>
+    <hyperlink ref="K18" r:id="rId27" display="https://www.4spe.org/i4a/pages/index.cfm?pageID=9239" xr:uid="{061FEADD-FD12-224D-BBEB-9E560D7996A9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>